<commit_message>
Included new files and repath some files
</commit_message>
<xml_diff>
--- a/python/Dados/Testes.xlsx
+++ b/python/Dados/Testes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Desktop\mba_dsa\python\Dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0DD7AAA-A919-4585-A974-AD8EDC8CFDF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D99734D-7E78-49B5-9EBE-35EDC5E63F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="29010" windowHeight="31785" xr2:uid="{6A0C2ABF-9AF9-4F78-8062-2AA66394EDC0}"/>
+    <workbookView xWindow="23880" yWindow="3075" windowWidth="33120" windowHeight="13365" xr2:uid="{6A0C2ABF-9AF9-4F78-8062-2AA66394EDC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -41,13 +41,13 @@
     <t>ID TEST</t>
   </si>
   <si>
-    <t>Velocidade</t>
+    <t>Talvez remover os primeiros 5s, pois foi necessário apertar o botão antes,TALVEZ FAZER ISSO PRA TODOS</t>
   </si>
   <si>
-    <t>Desbalanceado</t>
+    <t>Velocity</t>
   </si>
   <si>
-    <t>Talvez remover os primeiros 5s, pois foi necessário apertar o botão antes,TALVEZ FAZER ISSO PRA TODOS</t>
+    <t>Imbalance</t>
   </si>
 </sst>
 </file>
@@ -432,10 +432,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -548,7 +548,7 @@
         <v>0</v>
       </c>
       <c r="D11" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>